<commit_message>
Decision model: marketing-channel example, sensitivity analysis (+/-10%), CSV export
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/decision-model/decision-model.xlsx
+++ b/docs/decision-model/decision-model.xlsx
@@ -11,7 +11,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="المعايير والأوزان" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="تقييم البدائل" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="مصفوفة القرار" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="خطة التنفيذ والمتابعة" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="تحليل الحساسية" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="خطة التنفيذ والمتابعة" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -35,6 +36,9 @@
     </font>
     <font>
       <b val="1"/>
+    </font>
+    <font>
+      <i val="1"/>
     </font>
   </fonts>
   <fills count="3">
@@ -62,10 +66,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -80,6 +87,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -449,7 +457,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="70" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -465,52 +473,76 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>المشكلة</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>الحاجة إلى قناة تسويق رقمي لإطلاق منتج جديد بميزانية محدودة وجمهور مستهدف واضح.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>القرار المطلوب</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr"/>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>اختيار قناة التسويق الرقمي الأنسب لإطلاق المنتج.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>صاحب القرار</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr"/>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>[يُحدد لاحقًا]</t>
+        </is>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>تاريخ القرار</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr"/>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>[يُحدد لاحقًا]</t>
+        </is>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>القيود</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr"/>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>[يُحدد لاحقًا]</t>
+        </is>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>الافتراضات</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr"/>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>الدرجات على مقياس 1 إلى 10 حيث 10 = الأفضل، والمعايير مستقلة ومجموع أوزانها 1.00.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -523,7 +555,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -554,55 +586,66 @@
           <t>التكلفة</t>
         </is>
       </c>
-      <c r="B2" s="2" t="n">
-        <v>0.3</v>
+      <c r="B2" s="3" t="n">
+        <v>0.25</v>
       </c>
       <c r="C2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>السرعة</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="n">
-        <v>0.2</v>
+          <t>الوصول للجمهور المستهدف</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="n">
+        <v>0.3</v>
       </c>
       <c r="C3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>المخاطر</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="n">
-        <v>0.25</v>
+          <t>سرعة النتائج</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>0.2</v>
       </c>
       <c r="C4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>الأثر الاستراتيجي</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="n">
-        <v>0.25</v>
+          <t>قابلية القياس</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>0.15</v>
       </c>
       <c r="C5" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>الاستدامة</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
         <is>
           <t>المجموع</t>
         </is>
       </c>
-      <c r="B6" s="4">
-        <f>SUM(B2:B5)</f>
-        <v/>
-      </c>
-      <c r="C6" s="3" t="inlineStr"/>
+      <c r="B7" s="5">
+        <f>SUM(B2:B6)</f>
+        <v/>
+      </c>
+      <c r="C7" s="4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -615,10 +658,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
@@ -638,17 +681,17 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>البديل A</t>
+          <t>البديل مدفوعة</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>البديل B</t>
+          <t>البديل محتوى</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>البديل C</t>
+          <t>البديل مؤثرون</t>
         </is>
       </c>
     </row>
@@ -658,97 +701,117 @@
           <t>التكلفة</t>
         </is>
       </c>
-      <c r="B2" s="2">
+      <c r="B2" s="3">
         <f>'المعايير والأوزان'!B2</f>
         <v/>
       </c>
-      <c r="C2" s="5" t="n">
-        <v>8</v>
-      </c>
-      <c r="D2" s="5" t="n">
-        <v>7</v>
-      </c>
-      <c r="E2" s="5" t="n">
+      <c r="C2" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="D2" s="6" t="n">
         <v>9</v>
+      </c>
+      <c r="E2" s="6" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>السرعة</t>
-        </is>
-      </c>
-      <c r="B3" s="2">
+          <t>الوصول للجمهور المستهدف</t>
+        </is>
+      </c>
+      <c r="B3" s="3">
         <f>'المعايير والأوزان'!B3</f>
         <v/>
       </c>
-      <c r="C3" s="5" t="n">
-        <v>7</v>
-      </c>
-      <c r="D3" s="5" t="n">
+      <c r="C3" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="E3" s="5" t="n">
+      <c r="D3" s="6" t="n">
         <v>6</v>
+      </c>
+      <c r="E3" s="6" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>المخاطر</t>
-        </is>
-      </c>
-      <c r="B4" s="2">
+          <t>سرعة النتائج</t>
+        </is>
+      </c>
+      <c r="B4" s="3">
         <f>'المعايير والأوزان'!B4</f>
         <v/>
       </c>
-      <c r="C4" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="D4" s="5" t="n">
-        <v>8</v>
-      </c>
-      <c r="E4" s="5" t="n">
-        <v>5</v>
+      <c r="C4" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="D4" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="E4" s="6" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>الأثر الاستراتيجي</t>
-        </is>
-      </c>
-      <c r="B5" s="2">
+          <t>قابلية القياس</t>
+        </is>
+      </c>
+      <c r="B5" s="3">
         <f>'المعايير والأوزان'!B5</f>
         <v/>
       </c>
-      <c r="C5" s="5" t="n">
+      <c r="C5" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="D5" s="5" t="n">
-        <v>7</v>
-      </c>
-      <c r="E5" s="5" t="n">
-        <v>8</v>
+      <c r="D5" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="E5" s="6" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>الاستدامة</t>
+        </is>
+      </c>
+      <c r="B6" s="3">
+        <f>'المعايير والأوزان'!B6</f>
+        <v/>
+      </c>
+      <c r="C6" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="D6" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="E6" s="6" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
         <is>
           <t>الدرجة المرجحة</t>
         </is>
       </c>
-      <c r="B6" s="6" t="inlineStr"/>
-      <c r="C6" s="4">
-        <f>SUMPRODUCT($B$2:$B$5,C2:C5)</f>
-        <v/>
-      </c>
-      <c r="D6" s="4">
-        <f>SUMPRODUCT($B$2:$B$5,D2:D5)</f>
-        <v/>
-      </c>
-      <c r="E6" s="4">
-        <f>SUMPRODUCT($B$2:$B$5,E2:E5)</f>
+      <c r="B7" s="7" t="inlineStr"/>
+      <c r="C7" s="5">
+        <f>SUMPRODUCT($B$2:$B$6,C2:C6)</f>
+        <v/>
+      </c>
+      <c r="D7" s="5">
+        <f>SUMPRODUCT($B$2:$B$6,D2:D6)</f>
+        <v/>
+      </c>
+      <c r="E7" s="5">
+        <f>SUMPRODUCT($B$2:$B$6,E2:E6)</f>
         <v/>
       </c>
     </row>
@@ -766,7 +829,7 @@
   <dimension ref="A1:D4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
@@ -795,58 +858,58 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="B2" s="2">
-        <f>'تقييم البدائل'!C6</f>
-        <v/>
-      </c>
-      <c r="C2" s="5">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>مدفوعة</t>
+        </is>
+      </c>
+      <c r="B2" s="3">
+        <f>'تقييم البدائل'!C7</f>
+        <v/>
+      </c>
+      <c r="C2" s="6">
         <f>RANK(B2,$B$2:$B$4)</f>
         <v/>
       </c>
-      <c r="D2" s="5">
+      <c r="D2" s="6">
         <f>IF(C2=1,"✅ مختار","")</f>
         <v/>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="B3" s="2">
-        <f>'تقييم البدائل'!D6</f>
-        <v/>
-      </c>
-      <c r="C3" s="5">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>محتوى</t>
+        </is>
+      </c>
+      <c r="B3" s="3">
+        <f>'تقييم البدائل'!D7</f>
+        <v/>
+      </c>
+      <c r="C3" s="6">
         <f>RANK(B3,$B$2:$B$4)</f>
         <v/>
       </c>
-      <c r="D3" s="5">
+      <c r="D3" s="6">
         <f>IF(C3=1,"✅ مختار","")</f>
         <v/>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="B4" s="2">
-        <f>'تقييم البدائل'!E6</f>
-        <v/>
-      </c>
-      <c r="C4" s="5">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>مؤثرون</t>
+        </is>
+      </c>
+      <c r="B4" s="3">
+        <f>'تقييم البدائل'!E7</f>
+        <v/>
+      </c>
+      <c r="C4" s="6">
         <f>RANK(B4,$B$2:$B$4)</f>
         <v/>
       </c>
-      <c r="D4" s="5">
+      <c r="D4" s="6">
         <f>IF(C4=1,"✅ مختار","")</f>
         <v/>
       </c>
@@ -857,6 +920,356 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="8" t="inlineStr">
+        <is>
+          <t>تغيير كل وزن بنسبة ±10% ثم إعادة التطبيع إلى 1.00. قيم محسوبة بالسكربت.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>السيناريو</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>البديل مدفوعة</t>
+        </is>
+      </c>
+      <c r="C2" s="1" t="inlineStr">
+        <is>
+          <t>البديل محتوى</t>
+        </is>
+      </c>
+      <c r="D2" s="1" t="inlineStr">
+        <is>
+          <t>البديل مؤثرون</t>
+        </is>
+      </c>
+      <c r="E2" s="1" t="inlineStr">
+        <is>
+          <t>الفائز</t>
+        </is>
+      </c>
+      <c r="F2" s="1" t="inlineStr">
+        <is>
+          <t>تغيّر الفائز؟</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>الأساس</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="n">
+        <v>7.85</v>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>6.65</v>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>6.2</v>
+      </c>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>مدفوعة</t>
+        </is>
+      </c>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>لا</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>التكلفة -10%</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>7.9</v>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>6.59</v>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>6.23</v>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>مدفوعة</t>
+        </is>
+      </c>
+      <c r="F4" s="6" t="inlineStr">
+        <is>
+          <t>لا</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>التكلفة +10%</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>7.8</v>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>6.71</v>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>6.17</v>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>مدفوعة</t>
+        </is>
+      </c>
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>لا</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>الوصول للجمهور المستهدف -10%</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>7.81</v>
+      </c>
+      <c r="C6" s="3" t="n">
+        <v>6.67</v>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>6.14</v>
+      </c>
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t>مدفوعة</t>
+        </is>
+      </c>
+      <c r="F6" s="6" t="inlineStr">
+        <is>
+          <t>لا</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>الوصول للجمهور المستهدف +10%</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>7.88</v>
+      </c>
+      <c r="C7" s="3" t="n">
+        <v>6.63</v>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>6.25</v>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>مدفوعة</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="inlineStr">
+        <is>
+          <t>لا</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>سرعة النتائج -10%</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>7.83</v>
+      </c>
+      <c r="C8" s="3" t="n">
+        <v>6.7</v>
+      </c>
+      <c r="D8" s="3" t="n">
+        <v>6.18</v>
+      </c>
+      <c r="E8" s="6" t="inlineStr">
+        <is>
+          <t>مدفوعة</t>
+        </is>
+      </c>
+      <c r="F8" s="6" t="inlineStr">
+        <is>
+          <t>لا</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>سرعة النتائج +10%</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>7.87</v>
+      </c>
+      <c r="C9" s="3" t="n">
+        <v>6.6</v>
+      </c>
+      <c r="D9" s="3" t="n">
+        <v>6.22</v>
+      </c>
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>مدفوعة</t>
+        </is>
+      </c>
+      <c r="F9" s="6" t="inlineStr">
+        <is>
+          <t>لا</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>قابلية القياس -10%</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>7.83</v>
+      </c>
+      <c r="C10" s="3" t="n">
+        <v>6.66</v>
+      </c>
+      <c r="D10" s="3" t="n">
+        <v>6.22</v>
+      </c>
+      <c r="E10" s="6" t="inlineStr">
+        <is>
+          <t>مدفوعة</t>
+        </is>
+      </c>
+      <c r="F10" s="6" t="inlineStr">
+        <is>
+          <t>لا</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>قابلية القياس +10%</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>7.87</v>
+      </c>
+      <c r="C11" s="3" t="n">
+        <v>6.64</v>
+      </c>
+      <c r="D11" s="3" t="n">
+        <v>6.18</v>
+      </c>
+      <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t>مدفوعة</t>
+        </is>
+      </c>
+      <c r="F11" s="6" t="inlineStr">
+        <is>
+          <t>لا</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>الاستدامة -10%</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>7.88</v>
+      </c>
+      <c r="C12" s="3" t="n">
+        <v>6.63</v>
+      </c>
+      <c r="D12" s="3" t="n">
+        <v>6.22</v>
+      </c>
+      <c r="E12" s="6" t="inlineStr">
+        <is>
+          <t>مدفوعة</t>
+        </is>
+      </c>
+      <c r="F12" s="6" t="inlineStr">
+        <is>
+          <t>لا</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>الاستدامة +10%</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>7.82</v>
+      </c>
+      <c r="C13" s="3" t="n">
+        <v>6.67</v>
+      </c>
+      <c r="D13" s="3" t="n">
+        <v>6.18</v>
+      </c>
+      <c r="E13" s="6" t="inlineStr">
+        <is>
+          <t>مدفوعة</t>
+        </is>
+      </c>
+      <c r="F13" s="6" t="inlineStr">
+        <is>
+          <t>لا</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:F1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Decision model: one-way sweep with exact tipping points, cross-references, CSV 07-sweep
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/decision-model/decision-model.xlsx
+++ b/docs/decision-model/decision-model.xlsx
@@ -12,7 +12,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="تقييم البدائل" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="مصفوفة القرار" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="تحليل الحساسية" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="خطة التنفيذ والمتابعة" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="مسح الحساسية" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="خطة التنفيذ والمتابعة" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1275,6 +1276,478 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:N7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="12" max="12"/>
+    <col width="18" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="8" t="inlineStr">
+        <is>
+          <t>الخانات تُظهر الفائز عند كل وزن للمعيار، مع إعادة تطبيع بقية الأوزان تناسبيًا. نقطة الانقلاب محسوبة تحليليًا لأن الدرجات خطية في الوزن.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>المعيار</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>الوزن الحالي</t>
+        </is>
+      </c>
+      <c r="C2" s="1" t="inlineStr">
+        <is>
+          <t>0.05</t>
+        </is>
+      </c>
+      <c r="D2" s="1" t="inlineStr">
+        <is>
+          <t>0.10</t>
+        </is>
+      </c>
+      <c r="E2" s="1" t="inlineStr">
+        <is>
+          <t>0.15</t>
+        </is>
+      </c>
+      <c r="F2" s="1" t="inlineStr">
+        <is>
+          <t>0.20</t>
+        </is>
+      </c>
+      <c r="G2" s="1" t="inlineStr">
+        <is>
+          <t>0.25</t>
+        </is>
+      </c>
+      <c r="H2" s="1" t="inlineStr">
+        <is>
+          <t>0.30</t>
+        </is>
+      </c>
+      <c r="I2" s="1" t="inlineStr">
+        <is>
+          <t>0.35</t>
+        </is>
+      </c>
+      <c r="J2" s="1" t="inlineStr">
+        <is>
+          <t>0.40</t>
+        </is>
+      </c>
+      <c r="K2" s="1" t="inlineStr">
+        <is>
+          <t>0.45</t>
+        </is>
+      </c>
+      <c r="L2" s="1" t="inlineStr">
+        <is>
+          <t>0.50</t>
+        </is>
+      </c>
+      <c r="M2" s="1" t="inlineStr">
+        <is>
+          <t>نقطة الانقلاب</t>
+        </is>
+      </c>
+      <c r="N2" s="1" t="inlineStr">
+        <is>
+          <t>الفائز بعدها</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>التكلفة</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>0.25</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>مدفوعة</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>مدفوعة</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>مدفوعة</t>
+        </is>
+      </c>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>مدفوعة</t>
+        </is>
+      </c>
+      <c r="G3" s="6" t="inlineStr">
+        <is>
+          <t>مدفوعة</t>
+        </is>
+      </c>
+      <c r="H3" s="6" t="inlineStr">
+        <is>
+          <t>مدفوعة</t>
+        </is>
+      </c>
+      <c r="I3" s="6" t="inlineStr">
+        <is>
+          <t>مدفوعة</t>
+        </is>
+      </c>
+      <c r="J3" s="6" t="inlineStr">
+        <is>
+          <t>مدفوعة</t>
+        </is>
+      </c>
+      <c r="K3" s="6" t="inlineStr">
+        <is>
+          <t>مدفوعة</t>
+        </is>
+      </c>
+      <c r="L3" s="6" t="inlineStr">
+        <is>
+          <t>محتوى</t>
+        </is>
+      </c>
+      <c r="M3" s="6" t="inlineStr">
+        <is>
+          <t>0.464</t>
+        </is>
+      </c>
+      <c r="N3" s="6" t="inlineStr">
+        <is>
+          <t>محتوى</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>الوصول للجمهور المستهدف</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>0.30</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>مدفوعة</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>مدفوعة</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>مدفوعة</t>
+        </is>
+      </c>
+      <c r="F4" s="6" t="inlineStr">
+        <is>
+          <t>مدفوعة</t>
+        </is>
+      </c>
+      <c r="G4" s="6" t="inlineStr">
+        <is>
+          <t>مدفوعة</t>
+        </is>
+      </c>
+      <c r="H4" s="6" t="inlineStr">
+        <is>
+          <t>مدفوعة</t>
+        </is>
+      </c>
+      <c r="I4" s="6" t="inlineStr">
+        <is>
+          <t>مدفوعة</t>
+        </is>
+      </c>
+      <c r="J4" s="6" t="inlineStr">
+        <is>
+          <t>مدفوعة</t>
+        </is>
+      </c>
+      <c r="K4" s="6" t="inlineStr">
+        <is>
+          <t>مدفوعة</t>
+        </is>
+      </c>
+      <c r="L4" s="6" t="inlineStr">
+        <is>
+          <t>مدفوعة</t>
+        </is>
+      </c>
+      <c r="M4" s="6" t="inlineStr">
+        <is>
+          <t>لا يوجد ضمن 0–1</t>
+        </is>
+      </c>
+      <c r="N4" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>سرعة النتائج</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>0.20</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>مدفوعة</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>مدفوعة</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>مدفوعة</t>
+        </is>
+      </c>
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>مدفوعة</t>
+        </is>
+      </c>
+      <c r="G5" s="6" t="inlineStr">
+        <is>
+          <t>مدفوعة</t>
+        </is>
+      </c>
+      <c r="H5" s="6" t="inlineStr">
+        <is>
+          <t>مدفوعة</t>
+        </is>
+      </c>
+      <c r="I5" s="6" t="inlineStr">
+        <is>
+          <t>مدفوعة</t>
+        </is>
+      </c>
+      <c r="J5" s="6" t="inlineStr">
+        <is>
+          <t>مدفوعة</t>
+        </is>
+      </c>
+      <c r="K5" s="6" t="inlineStr">
+        <is>
+          <t>مدفوعة</t>
+        </is>
+      </c>
+      <c r="L5" s="6" t="inlineStr">
+        <is>
+          <t>مدفوعة</t>
+        </is>
+      </c>
+      <c r="M5" s="6" t="inlineStr">
+        <is>
+          <t>لا يوجد ضمن 0–1</t>
+        </is>
+      </c>
+      <c r="N5" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>قابلية القياس</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>0.15</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>مدفوعة</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>مدفوعة</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t>مدفوعة</t>
+        </is>
+      </c>
+      <c r="F6" s="6" t="inlineStr">
+        <is>
+          <t>مدفوعة</t>
+        </is>
+      </c>
+      <c r="G6" s="6" t="inlineStr">
+        <is>
+          <t>مدفوعة</t>
+        </is>
+      </c>
+      <c r="H6" s="6" t="inlineStr">
+        <is>
+          <t>مدفوعة</t>
+        </is>
+      </c>
+      <c r="I6" s="6" t="inlineStr">
+        <is>
+          <t>مدفوعة</t>
+        </is>
+      </c>
+      <c r="J6" s="6" t="inlineStr">
+        <is>
+          <t>مدفوعة</t>
+        </is>
+      </c>
+      <c r="K6" s="6" t="inlineStr">
+        <is>
+          <t>مدفوعة</t>
+        </is>
+      </c>
+      <c r="L6" s="6" t="inlineStr">
+        <is>
+          <t>مدفوعة</t>
+        </is>
+      </c>
+      <c r="M6" s="6" t="inlineStr">
+        <is>
+          <t>لا يوجد ضمن 0–1</t>
+        </is>
+      </c>
+      <c r="N6" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>الاستدامة</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>0.10</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>مدفوعة</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>مدفوعة</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>مدفوعة</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="inlineStr">
+        <is>
+          <t>مدفوعة</t>
+        </is>
+      </c>
+      <c r="G7" s="6" t="inlineStr">
+        <is>
+          <t>مدفوعة</t>
+        </is>
+      </c>
+      <c r="H7" s="6" t="inlineStr">
+        <is>
+          <t>مدفوعة</t>
+        </is>
+      </c>
+      <c r="I7" s="6" t="inlineStr">
+        <is>
+          <t>محتوى</t>
+        </is>
+      </c>
+      <c r="J7" s="6" t="inlineStr">
+        <is>
+          <t>محتوى</t>
+        </is>
+      </c>
+      <c r="K7" s="6" t="inlineStr">
+        <is>
+          <t>محتوى</t>
+        </is>
+      </c>
+      <c r="L7" s="6" t="inlineStr">
+        <is>
+          <t>محتوى</t>
+        </is>
+      </c>
+      <c r="M7" s="6" t="inlineStr">
+        <is>
+          <t>0.308</t>
+        </is>
+      </c>
+      <c r="N7" s="6" t="inlineStr">
+        <is>
+          <t>محتوى</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:N1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>

</xml_diff>

<commit_message>
Decision model: safety margin (exact, worst-case) and joint two-criteria tipping points
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/decision-model/decision-model.xlsx
+++ b/docs/decision-model/decision-model.xlsx
@@ -13,7 +13,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="مصفوفة القرار" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="تحليل الحساسية" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="مسح الحساسية" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="خطة التنفيذ والمتابعة" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="هامش الأمان والتحليل الثنائي" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="خطة التنفيذ والمتابعة" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1748,6 +1749,462 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:H16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="8" t="inlineStr">
+        <is>
+          <t>هامش الأمان: أكبر تغيير نسبي ±ε في كل الأوزان معًا يصمد أمامه الفائز. الانقلاب الثنائي: رفع وزني معيارين بمقدار t لكل منهما مع تطبيع البقية.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>المنافس</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>هامش الأمان ε*</t>
+        </is>
+      </c>
+      <c r="C2" s="1" t="inlineStr">
+        <is>
+          <t>أسوأ وزن: التكلفة</t>
+        </is>
+      </c>
+      <c r="D2" s="1" t="inlineStr">
+        <is>
+          <t>أسوأ وزن: الوصول للجمهور المستهدف</t>
+        </is>
+      </c>
+      <c r="E2" s="1" t="inlineStr">
+        <is>
+          <t>أسوأ وزن: سرعة النتائج</t>
+        </is>
+      </c>
+      <c r="F2" s="1" t="inlineStr">
+        <is>
+          <t>أسوأ وزن: قابلية القياس</t>
+        </is>
+      </c>
+      <c r="G2" s="1" t="inlineStr">
+        <is>
+          <t>أسوأ وزن: الاستدامة</t>
+        </is>
+      </c>
+      <c r="H2" s="1" t="inlineStr">
+        <is>
+          <t>الفارق عند أسوأ حالة</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>محتوى</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>34.3%</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>0.374</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>0.220</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>0.146</t>
+        </is>
+      </c>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>0.110</t>
+        </is>
+      </c>
+      <c r="G3" s="6" t="inlineStr">
+        <is>
+          <t>0.150</t>
+        </is>
+      </c>
+      <c r="H3" s="6" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>مؤثرون</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F4" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G4" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H4" s="6" t="inlineStr">
+        <is>
+          <t>لا ينقلب</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="n"/>
+      <c r="B5" s="6" t="n"/>
+      <c r="C5" s="6" t="n"/>
+      <c r="D5" s="6" t="n"/>
+      <c r="E5" s="6" t="n"/>
+      <c r="F5" s="6" t="n"/>
+      <c r="G5" s="6" t="n"/>
+      <c r="H5" s="6" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>المعيار الأول</t>
+        </is>
+      </c>
+      <c r="B6" s="1" t="inlineStr">
+        <is>
+          <t>المعيار الثاني</t>
+        </is>
+      </c>
+      <c r="C6" s="1" t="inlineStr">
+        <is>
+          <t>نقطة الانقلاب المشتركة t</t>
+        </is>
+      </c>
+      <c r="D6" s="1" t="inlineStr">
+        <is>
+          <t>الفائز بعدها</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="n"/>
+      <c r="F6" s="6" t="n"/>
+      <c r="G6" s="6" t="n"/>
+      <c r="H6" s="6" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>التكلفة</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>الوصول للجمهور المستهدف</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>لا يوجد</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="n"/>
+      <c r="F7" s="6" t="n"/>
+      <c r="G7" s="6" t="n"/>
+      <c r="H7" s="6" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>التكلفة</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>سرعة النتائج</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>لا يوجد</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E8" s="6" t="n"/>
+      <c r="F8" s="6" t="n"/>
+      <c r="G8" s="6" t="n"/>
+      <c r="H8" s="6" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>التكلفة</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>قابلية القياس</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>0.2400</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>محتوى</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="n"/>
+      <c r="F9" s="6" t="n"/>
+      <c r="G9" s="6" t="n"/>
+      <c r="H9" s="6" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>التكلفة</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>الاستدامة</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>0.0843</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>محتوى</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="n"/>
+      <c r="F10" s="6" t="n"/>
+      <c r="G10" s="6" t="n"/>
+      <c r="H10" s="6" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>الوصول للجمهور المستهدف</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>سرعة النتائج</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>لا يوجد</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="n"/>
+      <c r="F11" s="6" t="n"/>
+      <c r="G11" s="6" t="n"/>
+      <c r="H11" s="6" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>الوصول للجمهور المستهدف</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>قابلية القياس</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>لا يوجد</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E12" s="6" t="n"/>
+      <c r="F12" s="6" t="n"/>
+      <c r="G12" s="6" t="n"/>
+      <c r="H12" s="6" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>الوصول للجمهور المستهدف</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>الاستدامة</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>لا يوجد</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E13" s="6" t="n"/>
+      <c r="F13" s="6" t="n"/>
+      <c r="G13" s="6" t="n"/>
+      <c r="H13" s="6" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>سرعة النتائج</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>قابلية القياس</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>لا يوجد</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E14" s="6" t="n"/>
+      <c r="F14" s="6" t="n"/>
+      <c r="G14" s="6" t="n"/>
+      <c r="H14" s="6" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>سرعة النتائج</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>الاستدامة</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>لا يوجد</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E15" s="6" t="n"/>
+      <c r="F15" s="6" t="n"/>
+      <c r="G15" s="6" t="n"/>
+      <c r="H15" s="6" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>قابلية القياس</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>الاستدامة</t>
+        </is>
+      </c>
+      <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>0.2951</t>
+        </is>
+      </c>
+      <c r="D16" s="6" t="inlineStr">
+        <is>
+          <t>محتوى</t>
+        </is>
+      </c>
+      <c r="E16" s="6" t="n"/>
+      <c r="F16" s="6" t="n"/>
+      <c r="G16" s="6" t="n"/>
+      <c r="H16" s="6" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:G1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>

</xml_diff>